<commit_message>
R2: final numbers re-measured after merging main (only 21-6 moved: Quiet Contemplation, 41% -> 35%, still green)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R6XsJCmXvcJWh931mAnv4Q
</commit_message>
<xml_diff>
--- a/docs/road-curve-2026-10-19.xlsx
+++ b/docs/road-curve-2026-10-19.xlsx
@@ -14863,7 +14863,7 @@
         </is>
       </c>
       <c r="P156" t="n">
-        <v>40.8</v>
+        <v>35</v>
       </c>
       <c r="Q156" s="2" t="inlineStr">
         <is>
@@ -14871,7 +14871,7 @@
         </is>
       </c>
       <c r="R156" t="n">
-        <v>39.2</v>
+        <v>30.8</v>
       </c>
       <c r="S156" t="n">
         <v>42</v>
@@ -22109,10 +22109,10 @@
         <v>100</v>
       </c>
       <c r="G128" t="n">
-        <v>40.8</v>
+        <v>35</v>
       </c>
       <c r="H128" t="n">
-        <v>39.2</v>
+        <v>30.8</v>
       </c>
       <c r="I128" t="inlineStr">
         <is>

</xml_diff>